<commit_message>
chore(weekly-sync): auto-pull through 2026-07-02
</commit_message>
<xml_diff>
--- a/data/raw/inventory/Week 26/Tonor/Vendor SOH (SP-API).xlsx
+++ b/data/raw/inventory/Week 26/Tonor/Vendor SOH (SP-API).xlsx
@@ -571,12 +571,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FBA77101</t>
+          <t>FBA77103</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B07WLWN2ZT</t>
+          <t>B09Z5Q194D</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>TC-777</t>
+          <t>ORCA001</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -596,15 +596,15 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Tripod</t>
+          <t>Stand</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>1206</v>
+        <v>2412</v>
       </c>
       <c r="I3" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -619,13 +619,13 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="O3" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>68900.27</v>
+        <v>7528.69</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -636,12 +636,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FBA79578</t>
+          <t>FBA77104</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B0CFKZ72N7</t>
+          <t>B089SJGQBH</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -651,22 +651,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>TC20</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Dynamic Microphone</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Hand held Mic</t>
+          <t>Boom Arm Kit - XLR</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>1688</v>
+        <v>3015</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -699,12 +699,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FBA77103</t>
+          <t>FBA77105</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B09Z5Q194D</t>
+          <t>B089FVQD3Z</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ORCA001</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Stand</t>
+          <t>Boom Arm Kit</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>2412</v>
+        <v>1477</v>
       </c>
       <c r="I5" t="n">
         <v>2</v>
@@ -744,16 +744,16 @@
         <v>26</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>7528.69</v>
+        <v>3812.58</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -764,12 +764,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FBA79114</t>
+          <t>FBA79112</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B0CCV74CL7</t>
+          <t>B0BRKDLXCD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -779,25 +779,25 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TC310+</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Boom Arm Kit - USB - RGB</t>
+          <t>Boom Arm - RGB</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>1689</v>
+        <v>2412</v>
       </c>
       <c r="I6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -809,17 +809,15 @@
         <v>26</v>
       </c>
       <c r="M6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P6" t="n">
-        <v>14107.13</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
           <t>2026-06-27</t>
@@ -829,12 +827,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FBA79585</t>
+          <t>FBA77114</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B0CFKHCQ8W</t>
+          <t>B07TSN2H9D</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -844,25 +842,25 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>T20LP</t>
+          <t>TC-2030</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Low Profile Boom Arm</t>
+          <t>Boom Arm Kit - USB</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>845</v>
+        <v>4423</v>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -874,16 +872,16 @@
         <v>26</v>
       </c>
       <c r="M7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>4384.04</v>
+        <v>3890.39</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -894,12 +892,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FBA79576</t>
+          <t>FBA79111</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B0BRCR2QQ7</t>
+          <t>B0BRKFP94K</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -909,25 +907,25 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TC30S+</t>
+          <t>TD510</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Dynamic Microphone</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Boom Arm Kit + RGB</t>
+          <t>USB/XLR Mic</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>1749</v>
+        <v>2412</v>
       </c>
       <c r="I8" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -939,16 +937,16 @@
         <v>26</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8" t="n">
-        <v>14351.88</v>
+        <v>28003.99</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -959,12 +957,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FBA77116</t>
+          <t>FBA77115</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B0BBL47VR5</t>
+          <t>B08V1JS3NY</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -974,7 +972,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>TC40S</t>
+          <t>TC40</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -984,7 +982,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Boom Arm Kit - USB - RGB</t>
+          <t>Boom Arm Kit - USB</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -992,7 +990,7 @@
         <v>1930</v>
       </c>
       <c r="I9" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1004,16 +1002,16 @@
         <v>26</v>
       </c>
       <c r="M9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O9" t="n">
         <v>1</v>
       </c>
       <c r="P9" t="n">
-        <v>10345.5</v>
+        <v>25024.64</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1024,12 +1022,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FBA79115</t>
+          <t>FBA77101</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B0C8JDHLX9</t>
+          <t>B07WLWN2ZT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1039,25 +1037,25 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>TC-777</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Boom Arm Kit</t>
+          <t>Tripod</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>603</v>
+        <v>1206</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1072,13 +1070,13 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P10" t="n">
-        <v>2401.47</v>
+        <v>68900.27</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1089,12 +1087,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FBA79579</t>
+          <t>FBA77116</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>B0CQX4GVSB</t>
+          <t>B0BBL47VR5</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1104,25 +1102,25 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>TC40S</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Dynamic Microphone</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Hand held Mic</t>
+          <t>Boom Arm Kit - USB - RGB</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>1244</v>
+        <v>1930</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1134,15 +1132,17 @@
         <v>26</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>10345.5</v>
+      </c>
       <c r="Q11" t="inlineStr">
         <is>
           <t>2026-06-27</t>
@@ -1152,12 +1152,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FBA77106</t>
+          <t>FBA79574</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>B082W4B7SX</t>
+          <t>B0B4WTHLX5</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1167,25 +1167,25 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>TC30S</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Boom Arm Kit</t>
+          <t>Tripod+RGB</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>1164</v>
+        <v>1448</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1200,13 +1200,13 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>1652.04</v>
+        <v>15775.04</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1217,12 +1217,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FBA77111</t>
+          <t>FBA79116</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>B08CVP2HXP</t>
+          <t>B0BYHHSLPC</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>TC30</t>
+          <t>TC-777 PRO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1242,15 +1242,15 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Tripod</t>
+          <t>Tripod - RGB</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>1327</v>
+        <v>1086</v>
       </c>
       <c r="I13" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1262,16 +1262,16 @@
         <v>26</v>
       </c>
       <c r="M13" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="N13" t="n">
         <v>3</v>
       </c>
       <c r="O13" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="P13" t="n">
-        <v>156115.88</v>
+        <v>85703.7</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1282,12 +1282,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FBA79111</t>
+          <t>FBA79114</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>B0BRKFP94K</t>
+          <t>B0CCV74CL7</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1297,25 +1297,25 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>TD510</t>
+          <t>TC310+</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Dynamic Microphone</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>USB/XLR Mic</t>
+          <t>Boom Arm Kit - USB - RGB</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>2412</v>
+        <v>1689</v>
       </c>
       <c r="I14" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1327,16 +1327,16 @@
         <v>26</v>
       </c>
       <c r="M14" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="N14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P14" t="n">
-        <v>28003.99</v>
+        <v>14107.13</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1347,12 +1347,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FBA79112</t>
+          <t>FBA79585</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>B0BRKDLXCD</t>
+          <t>B0CFKHCQ8W</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T20LP</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1372,15 +1372,15 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Boom Arm - RGB</t>
+          <t>Low Profile Boom Arm</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>2412</v>
+        <v>845</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1392,15 +1392,17 @@
         <v>26</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="P15" t="n">
+        <v>4384.04</v>
+      </c>
       <c r="Q15" t="inlineStr">
         <is>
           <t>2026-06-27</t>
@@ -1410,12 +1412,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FBK77102</t>
+          <t>FBA79582</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>B07GVGMW59</t>
+          <t>B0CCVBQRFX</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1425,25 +1427,25 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>G11</t>
+          <t>TD510+</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Conference Microphone</t>
+          <t>Dynamic Microphone</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Wired</t>
+          <t>Hand held Mic + Boom Arm</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>1108</v>
+        <v>3491</v>
       </c>
       <c r="I16" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1455,16 +1457,16 @@
         <v>26</v>
       </c>
       <c r="M16" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>73079.14</v>
+        <v>4334.39</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1475,12 +1477,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FBA77117</t>
+          <t>FBA79576</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>B078WNW4YW</t>
+          <t>B0BRCR2QQ7</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1490,25 +1492,25 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>S20</t>
+          <t>TC30S+</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Microphone Isolation Shield</t>
+          <t>Boom Arm Kit + RGB</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>1174</v>
+        <v>1749</v>
       </c>
       <c r="I17" t="n">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1520,16 +1522,16 @@
         <v>26</v>
       </c>
       <c r="M17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="O17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>77996.81</v>
+        <v>14351.88</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -1540,12 +1542,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FBA79574</t>
+          <t>FBK77102</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>B0B4WTHLX5</t>
+          <t>B07GVGMW59</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1555,25 +1557,25 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TC30S</t>
+          <t>G11</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Conference Microphone</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Tripod+RGB</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>1448</v>
+        <v>1108</v>
       </c>
       <c r="I18" t="n">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1585,16 +1587,16 @@
         <v>26</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="N18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P18" t="n">
-        <v>15775.04</v>
+        <v>73079.14</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -1605,12 +1607,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FBA77115</t>
+          <t>FBA79697</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>B08V1JS3NY</t>
+          <t>B0CQX4K9P5</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1620,25 +1622,25 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>TC40</t>
+          <t>TD310</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Dynamic Microphone</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Boom Arm Kit - USB</t>
+          <t>Hand held Mic + Stand</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>1930</v>
+        <v>790</v>
       </c>
       <c r="I19" t="n">
-        <v>10</v>
+        <v>93</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1650,16 +1652,16 @@
         <v>26</v>
       </c>
       <c r="M19" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
         <v>2</v>
       </c>
-      <c r="O19" t="n">
-        <v>1</v>
-      </c>
       <c r="P19" t="n">
-        <v>25024.64</v>
+        <v>156590.89</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -1670,12 +1672,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FBA77113</t>
+          <t>FBA77106</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>B01ISNU3X4</t>
+          <t>B082W4B7SX</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1685,25 +1687,25 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Dynamic Microphone</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Hand held Mic</t>
+          <t>Boom Arm Kit</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>848</v>
+        <v>1164</v>
       </c>
       <c r="I20" t="n">
-        <v>233</v>
+        <v>1</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1715,16 +1717,16 @@
         <v>26</v>
       </c>
       <c r="M20" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>294646.16</v>
+        <v>1652.04</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -1735,12 +1737,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FBA77110</t>
+          <t>FBA79696</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>B08NDB5NWP</t>
+          <t>B0CQX3VB1R</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1750,25 +1752,25 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TM20</t>
+          <t>TD310+</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Conference Microphone</t>
+          <t>Dynamic Microphone</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Wired</t>
+          <t>Hand held Mic + Boom Arm</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>1695</v>
+        <v>927</v>
       </c>
       <c r="I21" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1780,16 +1782,16 @@
         <v>26</v>
       </c>
       <c r="M21" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P21" t="n">
-        <v>63652.13</v>
+        <v>61762.19</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -1800,12 +1802,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FBA79116</t>
+          <t>FBA77111</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>B0BYHHSLPC</t>
+          <t>B08CVP2HXP</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1815,7 +1817,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>TC-777 PRO</t>
+          <t>TC30</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1825,15 +1827,15 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Tripod - RGB</t>
+          <t>Tripod</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>1086</v>
+        <v>1327</v>
       </c>
       <c r="I22" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1845,16 +1847,16 @@
         <v>26</v>
       </c>
       <c r="M22" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="N22" t="n">
         <v>3</v>
       </c>
       <c r="O22" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="P22" t="n">
-        <v>85703.7</v>
+        <v>156115.88</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -1865,12 +1867,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FBA77114</t>
+          <t>FBA79579</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>B07TSN2H9D</t>
+          <t>B0CQX4GVSB</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1880,25 +1882,25 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>TC-2030</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Dynamic Microphone</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Boom Arm Kit - USB</t>
+          <t>Hand held Mic</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>4423</v>
+        <v>1244</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1913,14 +1915,12 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
-      <c r="P23" t="n">
-        <v>3890.39</v>
-      </c>
+      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
           <t>2026-06-27</t>
@@ -1930,12 +1930,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FBA79582</t>
+          <t>FBA77117</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>B0CCVBQRFX</t>
+          <t>B078WNW4YW</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1945,25 +1945,25 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>TD510+</t>
+          <t>S20</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Dynamic Microphone</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Hand held Mic + Boom Arm</t>
+          <t>Microphone Isolation Shield</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>3491</v>
+        <v>1174</v>
       </c>
       <c r="I24" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1978,13 +1978,13 @@
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P24" t="n">
-        <v>4334.39</v>
+        <v>77996.81</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -1995,12 +1995,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FBA77105</t>
+          <t>FBA79115</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>B089FVQD3Z</t>
+          <t>B0C8JDHLX9</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>1477</v>
+        <v>603</v>
       </c>
       <c r="I25" t="n">
         <v>2</v>
@@ -2040,16 +2040,16 @@
         <v>26</v>
       </c>
       <c r="M25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>3812.58</v>
+        <v>2401.47</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2060,12 +2060,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FBA79575</t>
+          <t>FBA79578</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>B0BG8CJXHH</t>
+          <t>B0CFKZ72N7</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2075,25 +2075,25 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>TC30+</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Dynamic Microphone</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Boom Arm Kit</t>
+          <t>Hand held Mic</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>1568</v>
+        <v>1688</v>
       </c>
       <c r="I26" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -2108,14 +2108,12 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
-      <c r="P26" t="n">
-        <v>22018.71</v>
-      </c>
+      <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr">
         <is>
           <t>2026-06-27</t>
@@ -2125,12 +2123,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FBA77104</t>
+          <t>FBA79575</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>B089SJGQBH</t>
+          <t>B0BG8CJXHH</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2140,7 +2138,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>TC20</t>
+          <t>TC30+</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2150,15 +2148,15 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Boom Arm Kit - XLR</t>
+          <t>Boom Arm Kit</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>3015</v>
+        <v>1568</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2173,12 +2171,14 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
-      <c r="P27" t="inlineStr"/>
+      <c r="P27" t="n">
+        <v>22018.71</v>
+      </c>
       <c r="Q27" t="inlineStr">
         <is>
           <t>2026-06-27</t>
@@ -2188,12 +2188,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FBA79697</t>
+          <t>FBA77113</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>B0CQX4K9P5</t>
+          <t>B01ISNU3X4</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>TD310</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2213,15 +2213,15 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Hand held Mic + Stand</t>
+          <t>Hand held Mic</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>790</v>
+        <v>848</v>
       </c>
       <c r="I28" t="n">
-        <v>93</v>
+        <v>233</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -2233,16 +2233,16 @@
         <v>26</v>
       </c>
       <c r="M28" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O28" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P28" t="n">
-        <v>156590.89</v>
+        <v>294646.16</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -2253,12 +2253,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>FBA79113</t>
+          <t>FBA77110</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>B0BTCXQQ6M</t>
+          <t>B08NDB5NWP</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2268,25 +2268,25 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>TC310</t>
+          <t>TM20</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Conference Microphone</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Tripod - RGB</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>1206</v>
+        <v>1695</v>
       </c>
       <c r="I29" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2298,16 +2298,16 @@
         <v>26</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>31520.85</v>
+        <v>63652.13</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -2318,12 +2318,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FBA79696</t>
+          <t>FBA79113</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>B0CQX3VB1R</t>
+          <t>B0BTCXQQ6M</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2333,25 +2333,25 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>TD310+</t>
+          <t>TC310</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Dynamic Microphone</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Hand held Mic + Boom Arm</t>
+          <t>Tripod - RGB</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>927</v>
+        <v>1206</v>
       </c>
       <c r="I30" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -2363,16 +2363,16 @@
         <v>26</v>
       </c>
       <c r="M30" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="O30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P30" t="n">
-        <v>61762.19</v>
+        <v>31520.85</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>

</xml_diff>